<commit_message>
add milestone on the assets
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template_v02.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template_v02.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="1" state="visible" r:id="rId2"/>
@@ -537,7 +537,7 @@
     <t xml:space="preserve">{texturing___sg_blocking_date}</t>
   </si>
   <si>
-    <t xml:space="preserve">mm/dd/yyyy</t>
+    <t xml:space="preserve">{shot_blocking_compositing}</t>
   </si>
   <si>
     <t xml:space="preserve">{lookdev___sg_final_date}</t>
@@ -3915,7 +3915,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="27.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="10.78"/>
@@ -3989,7 +3989,7 @@
       <c r="H3" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="33" t="s">
+      <c r="I3" s="31" t="s">
         <v>80</v>
       </c>
       <c r="J3" s="31" t="s">
@@ -4010,7 +4010,7 @@
       <c r="F4" s="32"/>
       <c r="G4" s="42"/>
       <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
+      <c r="I4" s="31"/>
       <c r="J4" s="42"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4052,7 +4052,9 @@
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H24" s="31"/>
+    </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>